<commit_message>
Movilidad interna rediseñada, unidades y series completas de Migracion, provincial de Ingresos v2
- Movilidad interna (PIDR b0cf8ffd): principal, quienes se mueven por
  nacionalidad y por sexo (96 cada una), nacionales por nacionalidad y por
  sexo (la de sexo es nueva) y lamina del glosario.
- Migracion: Movilidad interna y nacionales de la tasa neta por cada 1.000
  (PIDR 78c65713), mapas comunales de Movilidad incluidos; Migracion interna
  neta con las series completas 2019-2024.
- Provincial de Ingresos v2 (PIDR 260ce73d).

Fuera a proposito: el lote de Educacion (laminas por grupo, provinciales por
sexo y la evolucion nacional de E_REZMAT_a), en espera de la respuesta del
encargado de los datos, y dos XLSX de evolucion nacional regenerados con el.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/graficos_dimensiones/comunal_m_movinterna_a_2019_antofagasta.xlsx
+++ b/output/graficos_dimensiones/comunal_m_movinterna_a_2019_antofagasta.xlsx
@@ -69,7 +69,7 @@
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-27 22:04</t>
+    <t xml:space="preserve">2026-09-29 10:58</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>
@@ -505,7 +505,7 @@
         <v>2019</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>35.75</v>
+        <v>357.51</v>
       </c>
     </row>
     <row r="3">
@@ -522,7 +522,7 @@
         <v>2019</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>26.24</v>
+        <v>262.44</v>
       </c>
     </row>
     <row r="4">
@@ -539,7 +539,7 @@
         <v>2019</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>17.48</v>
+        <v>174.85</v>
       </c>
     </row>
     <row r="5">
@@ -556,7 +556,7 @@
         <v>2019</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>14.07</v>
+        <v>140.67</v>
       </c>
     </row>
     <row r="6">
@@ -573,7 +573,7 @@
         <v>2019</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>13.93</v>
+        <v>139.31</v>
       </c>
     </row>
     <row r="7">
@@ -590,7 +590,7 @@
         <v>2019</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>9.44</v>
+        <v>94.41</v>
       </c>
     </row>
     <row r="8">
@@ -607,7 +607,7 @@
         <v>2019</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>9.17</v>
+        <v>91.73</v>
       </c>
     </row>
     <row r="9">
@@ -624,7 +624,7 @@
         <v>2019</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>8</v>
+        <v>80.05</v>
       </c>
     </row>
     <row r="10">
@@ -641,7 +641,7 @@
         <v>2019</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>7.06</v>
+        <v>70.56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rezago 6 a 21 y Apoyo potencial nacionales, Movilidad con apellido en los titulos, payloads con version y html no-cache
</commit_message>
<xml_diff>
--- a/output/graficos_dimensiones/comunal_m_movinterna_a_2019_antofagasta.xlsx
+++ b/output/graficos_dimensiones/comunal_m_movinterna_a_2019_antofagasta.xlsx
@@ -69,7 +69,7 @@
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-29 10:58</t>
+    <t xml:space="preserve">2026-10-01 19:23</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>
@@ -87,7 +87,7 @@
     <t xml:space="preserve">Indicador</t>
   </si>
   <si>
-    <t xml:space="preserve">Movilidad interna (CMI)</t>
+    <t xml:space="preserve">Movilidad interna comunal (CMI)</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad territorial</t>

</xml_diff>